<commit_message>
final heatmap code update 8/20/26
</commit_message>
<xml_diff>
--- a/RAnalysis/Output/Yaquina_2009_2025/HYPOXIA_5_threshold_events_2026_0805_1029.xlsx
+++ b/RAnalysis/Output/Yaquina_2009_2025/HYPOXIA_5_threshold_events_2026_0805_1029.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\katie\Documents\BES_Internship\Seawater-Yaquina\RAnalysis\Output\Yaquina_2009_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008FBD04-C45A-4CB6-B3DF-D0FD40D90F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65E6B0E-0B9E-4903-AFE4-EA226D7C991E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BC41ECE1-8CF3-44A6-9828-EB94C554E057}"/>
+    <workbookView xWindow="396" yWindow="0" windowWidth="22644" windowHeight="13680" xr2:uid="{BC41ECE1-8CF3-44A6-9828-EB94C554E057}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="23">
   <si>
     <t>Year</t>
   </si>
@@ -448,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A724873D-B5F2-452E-B9DD-9C31EEEFBDCF}">
-  <dimension ref="A1:K205"/>
+  <dimension ref="A1:K193"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" customWidth="1"/>
@@ -6249,270 +6249,6 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A194">
-        <v>2025</v>
-      </c>
-      <c r="B194" t="s">
-        <v>10</v>
-      </c>
-      <c r="C194">
-        <v>5</v>
-      </c>
-      <c r="D194">
-        <v>0</v>
-      </c>
-      <c r="E194">
-        <v>0</v>
-      </c>
-      <c r="F194">
-        <v>0</v>
-      </c>
-      <c r="G194">
-        <v>0</v>
-      </c>
-      <c r="H194">
-        <v>6.48</v>
-      </c>
-      <c r="I194" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A195">
-        <v>2025</v>
-      </c>
-      <c r="B195" t="s">
-        <v>11</v>
-      </c>
-      <c r="C195">
-        <v>5</v>
-      </c>
-      <c r="D195">
-        <v>0</v>
-      </c>
-      <c r="E195">
-        <v>0</v>
-      </c>
-      <c r="F195">
-        <v>0</v>
-      </c>
-      <c r="G195">
-        <v>0</v>
-      </c>
-      <c r="H195">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="I195" t="e">
-        <f t="shared" ref="I195:I205" si="3">(D195*E195)/F195</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A196">
-        <v>2025</v>
-      </c>
-      <c r="B196" t="s">
-        <v>13</v>
-      </c>
-      <c r="C196">
-        <v>5</v>
-      </c>
-      <c r="D196">
-        <v>0</v>
-      </c>
-      <c r="E196">
-        <v>0</v>
-      </c>
-      <c r="F196">
-        <v>0</v>
-      </c>
-      <c r="G196">
-        <v>0</v>
-      </c>
-      <c r="H196">
-        <v>7.41</v>
-      </c>
-      <c r="I196" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A197">
-        <v>2025</v>
-      </c>
-      <c r="B197" t="s">
-        <v>14</v>
-      </c>
-      <c r="C197">
-        <v>5</v>
-      </c>
-      <c r="D197">
-        <v>0</v>
-      </c>
-      <c r="E197">
-        <v>0</v>
-      </c>
-      <c r="F197">
-        <v>0</v>
-      </c>
-      <c r="G197">
-        <v>5</v>
-      </c>
-      <c r="H197">
-        <v>8.39</v>
-      </c>
-      <c r="I197" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A198">
-        <v>2025</v>
-      </c>
-      <c r="B198" t="s">
-        <v>15</v>
-      </c>
-      <c r="C198">
-        <v>5</v>
-      </c>
-      <c r="G198">
-        <v>5</v>
-      </c>
-      <c r="I198" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A199">
-        <v>2025</v>
-      </c>
-      <c r="B199" t="s">
-        <v>16</v>
-      </c>
-      <c r="C199">
-        <v>5</v>
-      </c>
-      <c r="G199">
-        <v>5</v>
-      </c>
-      <c r="I199" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A200">
-        <v>2025</v>
-      </c>
-      <c r="B200" t="s">
-        <v>17</v>
-      </c>
-      <c r="C200">
-        <v>5</v>
-      </c>
-      <c r="G200">
-        <v>5</v>
-      </c>
-      <c r="I200" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A201">
-        <v>2025</v>
-      </c>
-      <c r="B201" t="s">
-        <v>18</v>
-      </c>
-      <c r="C201">
-        <v>5</v>
-      </c>
-      <c r="G201">
-        <v>5</v>
-      </c>
-      <c r="I201" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A202">
-        <v>2025</v>
-      </c>
-      <c r="B202" t="s">
-        <v>19</v>
-      </c>
-      <c r="C202">
-        <v>5</v>
-      </c>
-      <c r="G202">
-        <v>5</v>
-      </c>
-      <c r="I202" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A203">
-        <v>2025</v>
-      </c>
-      <c r="B203" t="s">
-        <v>20</v>
-      </c>
-      <c r="C203">
-        <v>5</v>
-      </c>
-      <c r="G203">
-        <v>5</v>
-      </c>
-      <c r="I203" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A204">
-        <v>2025</v>
-      </c>
-      <c r="B204" t="s">
-        <v>21</v>
-      </c>
-      <c r="C204">
-        <v>5</v>
-      </c>
-      <c r="G204">
-        <v>5</v>
-      </c>
-      <c r="I204" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A205">
-        <v>2025</v>
-      </c>
-      <c r="B205" t="s">
-        <v>22</v>
-      </c>
-      <c r="C205">
-        <v>5</v>
-      </c>
-      <c r="G205">
-        <v>5</v>
-      </c>
-      <c r="I205" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>